<commit_message>
Add QR/OCR scan modals
</commit_message>
<xml_diff>
--- a/shipped.xlsx
+++ b/shipped.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhiyongsong/warranty-h5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BFDF5D-9BF6-8847-A09C-790B2553BC12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52299135-B0CD-8044-8EC7-3403CB80F5DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="980" yWindow="1820" windowWidth="28100" windowHeight="17360" xr2:uid="{06E9EA4E-ACF2-7B48-B344-DC47D15C37B2}"/>
+    <workbookView xWindow="1040" yWindow="3720" windowWidth="39340" windowHeight="24720" xr2:uid="{06E9EA4E-ACF2-7B48-B344-DC47D15C37B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="76">
   <si>
     <t>AKSOB00691TAK</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -224,6 +224,75 @@
   </si>
   <si>
     <t>K100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A01460/LS1EMS01872</t>
+  </si>
+  <si>
+    <t>L100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01873</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01877</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01875</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01901</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01888</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01910</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01864</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01866</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01849</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01846</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01830</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01836</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01816</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01823</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01801</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01818</t>
+  </si>
+  <si>
+    <t>A01460/LS1ELU01806</t>
+  </si>
+  <si>
+    <t>A01461/LS1EKU00024</t>
+  </si>
+  <si>
+    <t>U100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AKSN700869TAK</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -270,13 +339,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -611,7 +681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31C950AE-A80A-E04D-BC1D-D1BD5062594E}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="28.1640625" customWidth="1"/>
@@ -637,7 +707,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
         <v>53</v>
@@ -651,7 +721,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
         <v>53</v>
@@ -665,7 +735,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
         <v>53</v>
@@ -679,7 +749,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
         <v>53</v>
@@ -693,7 +763,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
         <v>53</v>
@@ -707,7 +777,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
         <v>53</v>
@@ -721,7 +791,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
         <v>53</v>
@@ -735,7 +805,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
         <v>53</v>
@@ -749,7 +819,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
         <v>53</v>
@@ -763,7 +833,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B11" t="s">
         <v>53</v>
@@ -777,7 +847,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B12" t="s">
         <v>53</v>
@@ -791,7 +861,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
         <v>53</v>
@@ -805,7 +875,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
         <v>53</v>
@@ -819,7 +889,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s">
         <v>53</v>
@@ -833,7 +903,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B16" t="s">
         <v>53</v>
@@ -847,7 +917,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="B17" t="s">
         <v>53</v>
@@ -861,7 +931,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
         <v>53</v>
@@ -875,7 +945,7 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" t="s">
         <v>53</v>
@@ -889,7 +959,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B20" t="s">
         <v>53</v>
@@ -903,7 +973,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21" t="s">
         <v>53</v>
@@ -917,7 +987,7 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B22" t="s">
         <v>53</v>
@@ -931,7 +1001,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23" t="s">
         <v>53</v>
@@ -945,7 +1015,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
         <v>53</v>
@@ -959,7 +1029,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
         <v>53</v>
@@ -973,7 +1043,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" t="s">
         <v>53</v>
@@ -987,7 +1057,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B27" t="s">
         <v>53</v>
@@ -1001,7 +1071,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" t="s">
         <v>53</v>
@@ -1015,7 +1085,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B29" t="s">
         <v>53</v>
@@ -1029,7 +1099,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B30" t="s">
         <v>53</v>
@@ -1043,7 +1113,7 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B31" t="s">
         <v>53</v>
@@ -1057,7 +1127,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="B32" t="s">
         <v>53</v>
@@ -1071,7 +1141,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33" t="s">
         <v>53</v>
@@ -1085,7 +1155,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B34" t="s">
         <v>53</v>
@@ -1099,7 +1169,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B35" t="s">
         <v>53</v>
@@ -1113,7 +1183,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B36" t="s">
         <v>53</v>
@@ -1127,7 +1197,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="B37" t="s">
         <v>53</v>
@@ -1141,7 +1211,7 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B38" t="s">
         <v>53</v>
@@ -1155,7 +1225,7 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39" t="s">
         <v>53</v>
@@ -1169,7 +1239,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B40" t="s">
         <v>53</v>
@@ -1183,7 +1253,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B41" t="s">
         <v>53</v>
@@ -1197,7 +1267,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B42" t="s">
         <v>53</v>
@@ -1211,7 +1281,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B43" t="s">
         <v>53</v>
@@ -1225,7 +1295,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B44" t="s">
         <v>53</v>
@@ -1239,7 +1309,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B45" t="s">
         <v>53</v>
@@ -1253,7 +1323,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B46" t="s">
         <v>53</v>
@@ -1267,7 +1337,7 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B47" t="s">
         <v>53</v>
@@ -1281,7 +1351,7 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B48" t="s">
         <v>53</v>
@@ -1295,7 +1365,7 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B49" t="s">
         <v>53</v>
@@ -1309,16 +1379,296 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
+        <v>27</v>
+      </c>
+      <c r="B50" t="s">
+        <v>53</v>
+      </c>
+      <c r="C50" s="1">
+        <v>46023</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" t="s">
         <v>28</v>
       </c>
-      <c r="B50" t="s">
-        <v>53</v>
-      </c>
-      <c r="C50" s="1">
-        <v>46023</v>
-      </c>
-      <c r="D50">
-        <v>1</v>
+      <c r="B51" t="s">
+        <v>53</v>
+      </c>
+      <c r="C51" s="1">
+        <v>46023</v>
+      </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" t="s">
+        <v>55</v>
+      </c>
+      <c r="C52" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D52">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" t="s">
+        <v>55</v>
+      </c>
+      <c r="C53" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B54" t="s">
+        <v>55</v>
+      </c>
+      <c r="C54" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B55" t="s">
+        <v>55</v>
+      </c>
+      <c r="C55" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D55">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" t="s">
+        <v>55</v>
+      </c>
+      <c r="C56" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D56">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B57" t="s">
+        <v>55</v>
+      </c>
+      <c r="C57" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D57">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B58" t="s">
+        <v>55</v>
+      </c>
+      <c r="C58" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D58">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B59" t="s">
+        <v>55</v>
+      </c>
+      <c r="C59" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B60" t="s">
+        <v>55</v>
+      </c>
+      <c r="C60" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B61" t="s">
+        <v>55</v>
+      </c>
+      <c r="C61" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D61">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B62" t="s">
+        <v>55</v>
+      </c>
+      <c r="C62" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B63" t="s">
+        <v>55</v>
+      </c>
+      <c r="C63" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D63">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B64" t="s">
+        <v>55</v>
+      </c>
+      <c r="C64" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D64">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B65" t="s">
+        <v>55</v>
+      </c>
+      <c r="C65" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D65">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B66" t="s">
+        <v>55</v>
+      </c>
+      <c r="C66" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D66">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B67" t="s">
+        <v>55</v>
+      </c>
+      <c r="C67" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D67">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B68" t="s">
+        <v>55</v>
+      </c>
+      <c r="C68" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D68">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B69" t="s">
+        <v>55</v>
+      </c>
+      <c r="C69" s="1">
+        <v>45931</v>
+      </c>
+      <c r="D69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" t="s">
+        <v>73</v>
+      </c>
+      <c r="B70" t="s">
+        <v>74</v>
+      </c>
+      <c r="C70" s="1">
+        <v>45717</v>
+      </c>
+      <c r="D70">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>